<commit_message>
Merge Law, Politics of Aspiration and Power BI lexicons into one glossary each
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PTZNKtij4izWQRBJPfFcs4
</commit_message>
<xml_diff>
--- a/courses/law/Constitution-Law-Lexicon.xlsx
+++ b/courses/law/Constitution-Law-Lexicon.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Constitution &amp; Law Lexicon" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Constitution &amp; Law Lexicon" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Categories" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Constitution &amp; Law Lexicon'!$A$1:$F$66</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Constitution &amp; Law Lexicon'!$A$1:$F$96</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F66"/>
+  <dimension ref="A1:F96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -555,7 +555,7 @@
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>Judicial principle that Parliament cannot amend the Constitution to destroy its essential features. Established in Kesavananda Bharati v. State of Kerala (1973).</t>
+          <t>The doctrine that Parliament may amend the Constitution but cannot destroy its essential features, such as judicial review, federalism, and fundamental rights. It is the ultimate check on majoritarian rewriting of the constitutional bargain.</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
@@ -593,7 +593,7 @@
           <t>7,635 amendments debated across 165 days of deliberation</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr"/>
+      <c r="F3" s="9" t="n"/>
     </row>
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="2" t="n">
@@ -611,7 +611,7 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Introductory statement declaring India as sovereign, socialist, secular, democratic republic committed to justice, liberty, equality, fraternity. 'Socialist' and 'secular' added by 42nd Amendment (1976).</t>
+          <t>The opening declaration of the Constitution, describing India as a sovereign, socialist, secular, democratic republic committed to justice, liberty, equality, and fraternity. Courts treat it as the interpretive key to the whole document.</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -641,7 +641,7 @@
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>Ambedkar's concept requiring adherence to constitutional forms and processes over majoritarian social morality.</t>
+          <t>The principle that state action and social practice must conform to constitutional values — dignity, equality, fraternity — rather than to popular or majoritarian morality. Courts invoke it when social custom conflicts with rights.</t>
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr">
@@ -649,7 +649,7 @@
           <t>Navtej Singh Johar (2018), Sabarimala (2018)</t>
         </is>
       </c>
-      <c r="F5" s="9" t="inlineStr"/>
+      <c r="F5" s="9" t="n"/>
     </row>
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="2" t="n">
@@ -667,7 +667,7 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Divides legislative subjects into Union List (97+ items), State List (66 items), and Concurrent List (47 items). Central law prevails on concurrent subjects.</t>
+          <t>The division of lawmaking power between the Union, the States, and both jointly, through the Union, State, and Concurrent Lists. Knowing which list a subject sits in tells you which government to engage.</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -717,29 +717,25 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Article 14</t>
+          <t>Constitution of India</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Fundamental Rights</t>
+          <t>Constitutional Foundations</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Right to equality before the law and equal protection of the laws. Permits reasonable classification but prohibits arbitrary state action.</t>
+          <t>The supreme law of India, adopted on 26 November 1949 and in force since 26 January 1950. It establishes the structure of the state, guarantees rights, and sets the goals of social and economic justice that development practice operationalises.</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>E.P. Royappa (1974): arbitrariness is the antithesis of Article 14</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>Article 14</t>
-        </is>
-      </c>
+          <t>When a Dalit family is denied ration entitlements, a field worker can frame the denial not as a scheme failure but as a breach of constitutional guarantees of equality and dignity.</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="n"/>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="6" t="n">
@@ -747,29 +743,25 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Article 19</t>
+          <t>Fifth and Sixth Schedules</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>Fundamental Rights</t>
+          <t>Constitutional Foundations</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>Guarantees six freedoms: speech, assembly, association, movement, residence, profession. Subject to 'reasonable restrictions.'</t>
+          <t>Special constitutional regimes for tribal areas: the Fifth Schedule for Scheduled Areas in mainland states and the Sixth Schedule for autonomous councils in the Northeast. They restrict land alienation and give governors and councils special powers.</t>
         </is>
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>Shreya Singhal (2015): struck down Section 66A IT Act</t>
-        </is>
-      </c>
-      <c r="F9" s="9" t="inlineStr">
-        <is>
-          <t>Article 19(1)(a)-(g)</t>
-        </is>
-      </c>
+          <t>In the Samatha judgment (1997), the Supreme Court used Fifth Schedule protections to void mining leases to private companies on tribal land in Andhra Pradesh.</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="n"/>
     </row>
     <row r="10" ht="45" customHeight="1">
       <c r="A10" s="2" t="n">
@@ -777,7 +769,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Article 21</t>
+          <t>Article 14</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -787,17 +779,17 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Right to life and personal liberty. Expanded from narrow reading (A.K. Gopalan, 1950) to substantive due process (Maneka Gandhi, 1978).</t>
+          <t>The guarantee of equality before the law and equal protection of the laws. State action that is arbitrary, or classifies people without a reasonable basis linked to a legitimate purpose, violates Article 14.</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Now encompasses livelihood, shelter, education, health, environment, food, privacy, dignity</t>
+          <t>E.P. Royappa (1974): arbitrariness is the antithesis of Article 14</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>Article 21</t>
+          <t>Article 14</t>
         </is>
       </c>
     </row>
@@ -807,7 +799,7 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Article 32</t>
+          <t>Article 19</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
@@ -817,17 +809,17 @@
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>Right to constitutional remedies. Supreme Court can issue writs for enforcement of fundamental rights. Called 'soul of the Constitution' by Ambedkar.</t>
+          <t>Guarantees six freedoms: speech, assembly, association, movement, residence, profession. Subject to 'reasonable restrictions.'</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>PUCL v. UOI (2001): mid-day meals; T.N. Godavarman (1996): forest protection</t>
+          <t>Shreya Singhal (2015): struck down Section 66A IT Act</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>Article 32</t>
+          <t>Article 19(1)(a)-(g)</t>
         </is>
       </c>
     </row>
@@ -837,7 +829,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Writ Jurisdiction</t>
+          <t>Article 21</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -847,17 +839,17 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Power of Supreme Court (Art. 32) and High Courts (Art. 226) to issue prerogative writs: habeas corpus, mandamus, certiorari, prohibition, quo warranto.</t>
+          <t>The right to life and personal liberty, judicially expanded into the widest source of socio-economic rights: dignity, health, shelter, food, clean environment, and education. Most development-sector PILs are argued as Article 21 claims.</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Art. 226 is broader than Art. 32, extending to legal rights beyond fundamental rights</t>
+          <t>Now encompasses livelihood, shelter, education, health, environment, food, privacy, dignity</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Articles 32, 226</t>
+          <t>Article 21</t>
         </is>
       </c>
     </row>
@@ -867,7 +859,7 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Reasonable Restrictions</t>
+          <t>Article 32</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
@@ -877,17 +869,17 @@
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>Grounds on which Article 19 freedoms may be limited: sovereignty, security, public order, decency, morality, contempt, defamation, incitement.</t>
+          <t>Right to constitutional remedies. Supreme Court can issue writs for enforcement of fundamental rights. Called 'soul of the Constitution' by Ambedkar.</t>
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
-          <t>Courts apply proportionality test: narrowly tailored, legitimate aim, least restrictive means</t>
+          <t>PUCL v. UOI (2001): mid-day meals; T.N. Godavarman (1996): forest protection</t>
         </is>
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t>Article 19(2)-(6)</t>
+          <t>Article 32</t>
         </is>
       </c>
     </row>
@@ -897,7 +889,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Right to Privacy</t>
+          <t>Writ Jurisdiction</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -907,17 +899,17 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Recognized as fundamental right under Art. 21 in Puttaswamy (2017). Three-fold test: legality, legitimate aim, proportionality.</t>
+          <t>The power of the Supreme Court (Article 32) and High Courts (Article 226) to issue writs — habeas corpus, mandamus, certiorari, prohibition, quo warranto — to enforce rights. Article 226 is wider, covering legal as well as fundamental rights.</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Applied in Aadhaar judgment (2018): upheld for subsidies, struck down for private use</t>
+          <t>Art. 226 is broader than Art. 32, extending to legal rights beyond fundamental rights</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Article 21</t>
+          <t>Articles 32, 226</t>
         </is>
       </c>
     </row>
@@ -927,7 +919,7 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Untouchability Abolition</t>
+          <t>Reasonable Restrictions</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
@@ -937,17 +929,17 @@
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>Article 17 abolishes untouchability 'in any form.' One of few rights operating horizontally (binds private individuals).</t>
+          <t>Grounds on which Article 19 freedoms may be limited: sovereignty, security, public order, decency, morality, contempt, defamation, incitement.</t>
         </is>
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>Protection of Civil Rights Act (1955), SC/ST PoA Act (1989)</t>
+          <t>Courts apply proportionality test: narrowly tailored, legitimate aim, least restrictive means</t>
         </is>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>Article 17</t>
+          <t>Article 19(2)-(6)</t>
         </is>
       </c>
     </row>
@@ -957,7 +949,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Article 21A</t>
+          <t>Right to Privacy</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -967,17 +959,17 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Right to education for children aged 6-14. Inserted by 86th Amendment (2002). DPSP to fundamental right pathway.</t>
+          <t>Recognised as a fundamental right under Article 21 by a nine-judge bench, covering bodily, informational, and decisional privacy. State intrusions must pass a test of legality, necessity, and proportionality.</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Unni Krishnan (1993) read education into Art. 21; RTE Act (2009) implemented</t>
+          <t>Applied in Aadhaar judgment (2018): upheld for subsidies, struck down for private use</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Article 21A</t>
+          <t>Article 21</t>
         </is>
       </c>
     </row>
@@ -987,7 +979,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Article 300A</t>
+          <t>Untouchability Abolition</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
@@ -997,17 +989,17 @@
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>Right to property. Downgraded from fundamental to constitutional right by 44th Amendment (1978). Deprivation only by authority of law.</t>
+          <t>Article 17 abolishes untouchability 'in any form.' One of few rights operating horizontally (binds private individuals).</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>Land Acquisition Act 2013 replaced colonial 1894 Act</t>
+          <t>Protection of Civil Rights Act (1955), SC/ST PoA Act (1989)</t>
         </is>
       </c>
       <c r="F17" s="9" t="inlineStr">
         <is>
-          <t>Article 300A</t>
+          <t>Article 17</t>
         </is>
       </c>
     </row>
@@ -1017,27 +1009,27 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Directive Principles</t>
+          <t>Article 21A</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>State Policy &amp; Governance</t>
+          <t>Fundamental Rights</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Non-justiciable guidelines in Part IV directing the state toward social and economic justice.</t>
+          <t>Right to education for children aged 6-14. Inserted by 86th Amendment (2002). DPSP to fundamental right pathway.</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Art. 47 provided constitutional basis for NFSA (2013) covering 800 million people</t>
+          <t>Unni Krishnan (1993) read education into Art. 21; RTE Act (2009) implemented</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Articles 36-51</t>
+          <t>Article 21A</t>
         </is>
       </c>
     </row>
@@ -1047,27 +1039,27 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>DPSP-FR Harmonization</t>
+          <t>Article 300A</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>State Policy &amp; Governance</t>
+          <t>Fundamental Rights</t>
         </is>
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>Judicial doctrine that DPSPs and Fundamental Rights are complementary. Courts read DPSPs into expansive Art. 21 interpretation.</t>
+          <t>Right to property. Downgraded from fundamental to constitutional right by 44th Amendment (1978). Deprivation only by authority of law.</t>
         </is>
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>Right to education: DPSP Art. 45 to Art. 21 (Unni Krishnan, 1993) to Art. 21A (2002)</t>
+          <t>Land Acquisition Act 2013 replaced colonial 1894 Act</t>
         </is>
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
-          <t>Parts III and IV</t>
+          <t>Article 300A</t>
         </is>
       </c>
     </row>
@@ -1077,29 +1069,25 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Fundamental Duties</t>
+          <t>Fundamental Rights</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>State Policy &amp; Governance</t>
+          <t>Fundamental Rights</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Part IVA (Art. 51A), 42nd Amendment. Eleven duties including respecting Constitution, promoting harmony, protecting environment.</t>
+          <t>The justiciable rights in Part III (Articles 12-35), including equality, freedoms, life and liberty, and protection from exploitation. Unlike policy promises, these can be directly enforced in the Supreme Court and High Courts.</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>Used to support restrictions on animal sacrifice and environmental destruction</t>
-        </is>
-      </c>
-      <c r="F20" s="5" t="inlineStr">
-        <is>
-          <t>Article 51A</t>
-        </is>
-      </c>
+          <t>A bonded labour rescue relies on Article 23 (prohibition of forced labour) — a Fundamental Right enforceable against private employers, not just the state.</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="n"/>
     </row>
     <row r="21" ht="45" customHeight="1">
       <c r="A21" s="6" t="n">
@@ -1107,29 +1095,25 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Panchayati Raj</t>
+          <t>Right to Livelihood</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>State Policy &amp; Governance</t>
+          <t>Fundamental Rights</t>
         </is>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>Three-tier local self-governance constitutionalized by 73rd Amendment (1992). Reserved seats for SC/ST and women (min. one-third).</t>
+          <t>The judicial reading of Article 21 that livelihood is an integral facet of the right to life, so the state cannot deprive people of their means of living without fair procedure. It is the constitutional anchor for anti-eviction and vendor-rights work.</t>
         </is>
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>2.5 lakh+ gram panchayats, ~14 lakh elected women representatives</t>
-        </is>
-      </c>
-      <c r="F21" s="9" t="inlineStr">
-        <is>
-          <t>Articles 243-243O</t>
-        </is>
-      </c>
+          <t>In Olga Tellis v Bombay Municipal Corporation (1985), pavement dwellers won the principle that eviction without notice and hearing violates Article 21 because it extinguishes livelihood.</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="n"/>
     </row>
     <row r="22" ht="45" customHeight="1">
       <c r="A22" s="2" t="n">
@@ -1137,7 +1121,7 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Finance Commission</t>
+          <t>Directive Principles</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
@@ -1147,17 +1131,17 @@
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Constitutional body (Art. 280) recommending tax revenue distribution. 15th FC recommended 41% devolution to states.</t>
+          <t>Part IV goals — livelihood, living wages, nutrition, health, free legal aid — that are not directly enforceable in court but are fundamental to governance. Much of India’s welfare legislation converts these principles into statutory rights.</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>14th FC increased devolution from 32% to 42%, transforming Centre-state finances</t>
+          <t>Art. 47 provided constitutional basis for NFSA (2013) covering 800 million people</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Article 280</t>
+          <t>Articles 36-51</t>
         </is>
       </c>
     </row>
@@ -1167,7 +1151,7 @@
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Article 356</t>
+          <t>DPSP-FR Harmonization</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
@@ -1177,17 +1161,17 @@
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>President's Rule: central takeover on constitutional machinery failure. Used 100+ times. S.R. Bommai (1994) made it judicially reviewable.</t>
+          <t>Judicial doctrine that DPSPs and Fundamental Rights are complementary. Courts read DPSPs into expansive Art. 21 interpretation.</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
-          <t>Bommai: floor of legislature, not Governor's assessment, determines majority</t>
+          <t>Right to education: DPSP Art. 45 to Art. 21 (Unni Krishnan, 1993) to Art. 21A (2002)</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>Article 356</t>
+          <t>Parts III and IV</t>
         </is>
       </c>
     </row>
@@ -1197,7 +1181,7 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Fiscal Federalism</t>
+          <t>Fundamental Duties</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
@@ -1207,17 +1191,17 @@
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Framework for sharing financial resources between Centre and states through Finance Commission, GST Council, and centrally sponsored schemes.</t>
+          <t>Part IVA (Art. 51A), 42nd Amendment. Eleven duties including respecting Constitution, promoting harmony, protecting environment.</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>101st Amendment (2016) created GST Council for joint Centre-state tax decisions</t>
+          <t>Used to support restrictions on animal sacrifice and environmental destruction</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>Articles 268-281</t>
+          <t>Article 51A</t>
         </is>
       </c>
     </row>
@@ -1227,7 +1211,7 @@
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Anti-Defection Law</t>
+          <t>Panchayati Raj</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
@@ -1237,17 +1221,17 @@
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>Tenth Schedule (52nd Amendment, 1985): disqualifies legislators who defect. Speaker decides petitions, raising bias concerns.</t>
+          <t>Three-tier local self-governance constitutionalized by 73rd Amendment (1992). Reserved seats for SC/ST and women (min. one-third).</t>
         </is>
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>Kihoto Hollohan (1992): upheld but noted concerns about Speaker's dual role</t>
+          <t>2.5 lakh+ gram panchayats, ~14 lakh elected women representatives</t>
         </is>
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>Tenth Schedule</t>
+          <t>Articles 243-243O</t>
         </is>
       </c>
     </row>
@@ -1257,27 +1241,27 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Public Interest Litigation</t>
+          <t>Finance Commission</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Judicial System</t>
+          <t>State Policy &amp; Governance</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Innovation allowing any person to approach courts on behalf of those unable. Relaxed locus standi. Pioneered by Justices Bhagwati and Krishna Iyer.</t>
+          <t>Constitutional body (Art. 280) recommending tax revenue distribution. 15th FC recommended 41% devolution to states.</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>Hussainara Khatoon (1979): undertrial rights; Olga Tellis (1985): pavement dwellers' livelihood</t>
+          <t>14th FC increased devolution from 32% to 42%, transforming Centre-state finances</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>Articles 32, 226</t>
+          <t>Article 280</t>
         </is>
       </c>
     </row>
@@ -1287,27 +1271,27 @@
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Collegium System</t>
+          <t>Article 356</t>
         </is>
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>Judicial System</t>
+          <t>State Policy &amp; Governance</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>Judicial appointment mechanism: CJI and four senior judges recommend appointments. Established by Second (1993) and Third (1998) Judges Cases.</t>
+          <t>President's Rule: central takeover on constitutional machinery failure. Used 100+ times. S.R. Bommai (1994) made it judicially reviewable.</t>
         </is>
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>NJAC (99th Amendment, 2015) struck down as violating judicial independence (basic structure)</t>
+          <t>Bommai: floor of legislature, not Governor's assessment, determines majority</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>Article 124</t>
+          <t>Article 356</t>
         </is>
       </c>
     </row>
@@ -1317,27 +1301,27 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Judicial Review</t>
+          <t>Fiscal Federalism</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Judicial System</t>
+          <t>State Policy &amp; Governance</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Power of courts to examine legislative and executive action for constitutional validity. Part of basic structure (L. Chandra Kumar, 1997).</t>
+          <t>Framework for sharing financial resources between Centre and states through Finance Commission, GST Council, and centrally sponsored schemes.</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>Over 100 laws struck down, from sedition provisions to privacy violations</t>
+          <t>101st Amendment (2016) created GST Council for joint Centre-state tax decisions</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>Articles 13, 32, 226, 136</t>
+          <t>Articles 268-281</t>
         </is>
       </c>
     </row>
@@ -1347,25 +1331,29 @@
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Pendency Crisis</t>
+          <t>Anti-Defection Law</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>Judicial System</t>
+          <t>State Policy &amp; Governance</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>5+ crore cases pending: ~80,000 in SC, ~60 lakh in HCs, ~4.4 crore in district courts. 21 judges per million (UK: 51, Germany: 100+).</t>
+          <t>Tenth Schedule (52nd Amendment, 1985): disqualifies legislators who defect. Speaker decides petitions, raising bias concerns.</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>Average disposal time exceeds 3-5 years in many jurisdictions</t>
-        </is>
-      </c>
-      <c r="F29" s="9" t="inlineStr"/>
+          <t>Kihoto Hollohan (1992): upheld but noted concerns about Speaker's dual role</t>
+        </is>
+      </c>
+      <c r="F29" s="9" t="inlineStr">
+        <is>
+          <t>Tenth Schedule</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="45" customHeight="1">
       <c r="A30" s="2" t="n">
@@ -1373,7 +1361,7 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Lok Adalat</t>
+          <t>Public Interest Litigation</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
@@ -1383,17 +1371,17 @@
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>People's courts under Legal Services Authorities Act (1987). Conciliation-based. Decisions binding, final, non-appealable. No court fees.</t>
+          <t>A distinctly Indian procedure allowing any public-spirited person to move the courts on behalf of those unable to do so themselves, with relaxed standing and flexible remedies. It converted constitutional courts into a forum for the poor.</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>1.87 crore+ cases settled annually</t>
+          <t>Hussainara Khatoon (1979): undertrial rights; Olga Tellis (1985): pavement dwellers' livelihood</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>Article 39A</t>
+          <t>Articles 32, 226</t>
         </is>
       </c>
     </row>
@@ -1403,7 +1391,7 @@
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>Gram Nyayalaya</t>
+          <t>Collegium System</t>
         </is>
       </c>
       <c r="C31" s="8" t="inlineStr">
@@ -1413,15 +1401,19 @@
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>Village courts under Gram Nyayalayas Act (2008) at panchayat level. Only ~500 functioning by 2023 against target of thousands.</t>
+          <t>Judicial appointment mechanism: CJI and four senior judges recommend appointments. Established by Second (1993) and Third (1998) Judges Cases.</t>
         </is>
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>Persistent gap between legislative intent and implementation in access to justice</t>
-        </is>
-      </c>
-      <c r="F31" s="9" t="inlineStr"/>
+          <t>NJAC (99th Amendment, 2015) struck down as violating judicial independence (basic structure)</t>
+        </is>
+      </c>
+      <c r="F31" s="9" t="inlineStr">
+        <is>
+          <t>Article 124</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="45" customHeight="1">
       <c r="A32" s="2" t="n">
@@ -1429,7 +1421,7 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>PIL Abuse</t>
+          <t>Judicial Review</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
@@ -1439,15 +1431,19 @@
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Criticism that PIL has been captured by elite interests. Documented by Bhuwania in 'Courting the People' (2017).</t>
+          <t>The power of constitutional courts to strike down legislation and executive action that violate the Constitution. It is itself part of the basic structure and the reason rights on paper can be enforced in practice.</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>SC has imposed costs on frivolous petitioners, warning against 'publicity interest litigation'</t>
-        </is>
-      </c>
-      <c r="F32" s="5" t="inlineStr"/>
+          <t>Over 100 laws struck down, from sedition provisions to privacy violations</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>Articles 13, 32, 226, 136</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="45" customHeight="1">
       <c r="A33" s="6" t="n">
@@ -1455,29 +1451,25 @@
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>Reservation Policy</t>
+          <t>Pendency Crisis</t>
         </is>
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>Social Justice</t>
+          <t>Judicial System</t>
         </is>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>Affirmative action through Arts. 15(4), 16(4), 330, 332 for SC, ST, OBC in education, employment, legislatures.</t>
+          <t>5+ crore cases pending: ~80,000 in SC, ~60 lakh in HCs, ~4.4 crore in district courts. 21 judges per million (UK: 51, Germany: 100+).</t>
         </is>
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>Indra Sawhney (1992): 50% ceiling, creamy layer exclusion for OBCs</t>
-        </is>
-      </c>
-      <c r="F33" s="9" t="inlineStr">
-        <is>
-          <t>Articles 15(4), 16(4)</t>
-        </is>
-      </c>
+          <t>Average disposal time exceeds 3-5 years in many jurisdictions</t>
+        </is>
+      </c>
+      <c r="F33" s="9" t="n"/>
     </row>
     <row r="34" ht="45" customHeight="1">
       <c r="A34" s="2" t="n">
@@ -1485,25 +1477,29 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Creamy Layer</t>
+          <t>Lok Adalat</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Social Justice</t>
+          <t>Judicial System</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Economic threshold above which OBC individuals excluded from reservation. Currently Rs. 8 lakh. Does not apply to SC/ST.</t>
+          <t>A statutory forum where pending or pre-litigation disputes are settled by conciliation; its award has the force of a civil court decree and no court fee applies. It is fast but settlement-driven, so power imbalances need watching.</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>Introduced in Indra Sawhney (1992) to ensure benefits reach most disadvantaged OBCs</t>
-        </is>
-      </c>
-      <c r="F34" s="5" t="inlineStr"/>
+          <t>1.87 crore+ cases settled annually</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>Article 39A</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="45" customHeight="1">
       <c r="A35" s="6" t="n">
@@ -1511,29 +1507,25 @@
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>EWS Reservation</t>
+          <t>Gram Nyayalaya</t>
         </is>
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>Social Justice</t>
+          <t>Judicial System</t>
         </is>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>10% for Economically Weaker Sections among unreserved categories. 103rd Amendment (2019). Upheld in Janhit Abhiyan (2022), 3:2.</t>
+          <t>Village courts under Gram Nyayalayas Act (2008) at panchayat level. Only ~500 functioning by 2023 against target of thousands.</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
         <is>
-          <t>First economic-only reservation in Indian constitutional history</t>
-        </is>
-      </c>
-      <c r="F35" s="9" t="inlineStr">
-        <is>
-          <t>Article 15(6), 16(6)</t>
-        </is>
-      </c>
+          <t>Persistent gap between legislative intent and implementation in access to justice</t>
+        </is>
+      </c>
+      <c r="F35" s="9" t="n"/>
     </row>
     <row r="36" ht="45" customHeight="1">
       <c r="A36" s="2" t="n">
@@ -1541,25 +1533,25 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Sub-Classification of SCs</t>
+          <t>PIL Abuse</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Social Justice</t>
+          <t>Judicial System</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>States may create sub-categories within SCs for preferential treatment. Permitted in State of Punjab v. Davinder Singh (2024).</t>
+          <t>Criticism that PIL has been captured by elite interests. Documented by Bhuwania in 'Courting the People' (2017).</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>Allows prioritizing Valmikis, Mazhabi Sikhs, Arunthathiyars within SC category</t>
-        </is>
-      </c>
-      <c r="F36" s="5" t="inlineStr"/>
+          <t>SC has imposed costs on frivolous petitioners, warning against 'publicity interest litigation'</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="n"/>
     </row>
     <row r="37" ht="45" customHeight="1">
       <c r="A37" s="6" t="n">
@@ -1567,29 +1559,25 @@
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>Political Reservation</t>
+          <t>Locus Standi</t>
         </is>
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t>Social Justice</t>
+          <t>Judicial System</t>
         </is>
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>Reserved seats in Parliament and state legislatures for SC/ST proportional to population. Extended to 2030.</t>
+          <t>The requirement that a petitioner must have a direct legal interest in a dispute to be heard. PIL relaxed this rule so that NGOs and citizens can litigate on behalf of affected communities.</t>
         </is>
       </c>
       <c r="E37" s="9" t="inlineStr">
         <is>
-          <t>Pande (2003, AER): increased targeted public goods spending in SC-reserved constituencies</t>
-        </is>
-      </c>
-      <c r="F37" s="9" t="inlineStr">
-        <is>
-          <t>Articles 330-333</t>
-        </is>
-      </c>
+          <t>Bandhua Mukti Morcha, an NGO, was granted standing to petition for the release of bonded quarry workers it had no personal stake in — impossible under strict locus standi.</t>
+        </is>
+      </c>
+      <c r="F37" s="9" t="n"/>
     </row>
     <row r="38" ht="45" customHeight="1">
       <c r="A38" s="2" t="n">
@@ -1597,25 +1585,25 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>RTI Act</t>
+          <t>Habeas Corpus</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Rights-Based Legislation</t>
+          <t>Judicial System</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Right to Information Act (2005). Citizens can request information from public authorities within 30 days. Penalties: Rs. 250/day.</t>
+          <t>The writ commanding that a detained person be produced before the court and the legality of the detention justified. It is the classic remedy against illegal custody, trafficking, and bonded labour.</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>40-60 lakh applications annually. Peisakhin &amp; Pinto (2010): RTI reduced bureaucratic delays</t>
-        </is>
-      </c>
-      <c r="F38" s="5" t="inlineStr"/>
+          <t>Anti-trafficking organisations file habeas corpus petitions to produce girls confined in unlicensed shelter homes or employers’ houses.</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="n"/>
     </row>
     <row r="39" ht="45" customHeight="1">
       <c r="A39" s="6" t="n">
@@ -1623,29 +1611,25 @@
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>MGNREGA</t>
+          <t>Mandamus</t>
         </is>
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t>Rights-Based Legislation</t>
+          <t>Judicial System</t>
         </is>
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>100 days wage employment guarantee per rural household per year. Demand-driven with unemployment allowance.</t>
+          <t>The writ directing a public authority to perform a duty the law obliges it to perform. It is the workhorse remedy when officials simply fail to act on entitlements.</t>
         </is>
       </c>
       <c r="E39" s="9" t="inlineStr">
         <is>
-          <t>Imbert &amp; Papp (2015, AER): raised private-sector wages by 4.7%. Muralidharan et al. (2016): biometrics reduced leakage 40%</t>
-        </is>
-      </c>
-      <c r="F39" s="9" t="inlineStr">
-        <is>
-          <t>Article 41 (DPSP)</t>
-        </is>
-      </c>
+          <t>A High Court issues mandamus directing a municipal corporation to constitute the Town Vending Committee it has ignored for years under the Street Vendors Act.</t>
+        </is>
+      </c>
+      <c r="F39" s="9" t="n"/>
     </row>
     <row r="40" ht="45" customHeight="1">
       <c r="A40" s="2" t="n">
@@ -1653,25 +1637,25 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Forest Rights Act</t>
+          <t>Continuing Mandamus</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Rights-Based Legislation</t>
+          <t>Judicial System</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>Recognition of individual and community rights over forest land occupied before December 2005 for scheduled tribes and traditional forest dwellers.</t>
+          <t>A PIL innovation in which the court keeps a case open and issues rolling directions, monitoring compliance over months or years instead of passing one final order. It turns litigation into supervised implementation.</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>Section 4(5): Gram Sabha consent required before forest land diversion</t>
-        </is>
-      </c>
-      <c r="F40" s="5" t="inlineStr"/>
+          <t>In the right-to-food case, the Supreme Court appointed commissioners and monitored state compliance with its interim orders for over a decade.</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="n"/>
     </row>
     <row r="41" ht="45" customHeight="1">
       <c r="A41" s="6" t="n">
@@ -1679,29 +1663,25 @@
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>RTE Act</t>
+          <t>Natural Justice</t>
         </is>
       </c>
       <c r="C41" s="8" t="inlineStr">
         <is>
-          <t>Rights-Based Legislation</t>
+          <t>Judicial System</t>
         </is>
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>Free and compulsory education for ages 6-14. 25% reservation in private unaided schools for disadvantaged children.</t>
+          <t>The twin common-law principles that no one may be condemned unheard (audi alteram partem) and no one may judge their own cause (nemo judex in causa sua). Administrative decisions taken in breach are liable to be quashed.</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>ASER 2023: near-universal enrollment but only 65% of Grade 5 children read Grade 2 text</t>
-        </is>
-      </c>
-      <c r="F41" s="9" t="inlineStr">
-        <is>
-          <t>Article 21A</t>
-        </is>
-      </c>
+          <t>Cancelling a ration card or deregistering an anganwadi helper without notice and a hearing violates natural justice and can be set aside in a writ.</t>
+        </is>
+      </c>
+      <c r="F41" s="9" t="n"/>
     </row>
     <row r="42" ht="45" customHeight="1">
       <c r="A42" s="2" t="n">
@@ -1709,29 +1689,25 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>NFSA</t>
+          <t>Due Process</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Rights-Based Legislation</t>
+          <t>Judicial System</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>Subsidized foodgrains (rice Rs. 3/kg, wheat Rs. 2/kg) to ~800 million people through PDS.</t>
+          <t>The requirement, read into Article 21 after Maneka Gandhi, that any procedure affecting life or liberty must be fair, just, and reasonable — not merely enacted. Substantively unfair laws and arbitrary procedures both fail the test.</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>Dreze &amp; Khera (2017): PDS reform improved delivery but created exclusion errors</t>
-        </is>
-      </c>
-      <c r="F42" s="5" t="inlineStr">
-        <is>
-          <t>Article 47 (DPSP)</t>
-        </is>
-      </c>
+          <t>Demolition of homes without notice, hearing, or rehabilitation is challenged as a due-process violation, drawing on Olga Tellis and later slum-demolition jurisprudence.</t>
+        </is>
+      </c>
+      <c r="F42" s="5" t="n"/>
     </row>
     <row r="43" ht="45" customHeight="1">
       <c r="A43" s="6" t="n">
@@ -1739,25 +1715,25 @@
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>Social Audit</t>
+          <t>Legal Aid</t>
         </is>
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t>Rights-Based Legislation</t>
+          <t>Judicial System</t>
         </is>
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>Community-led verification of government records by beneficiaries. Mandated under MGNREGA since 2011.</t>
+          <t>The constitutional commitment (Article 39A) to free legal services for the poor, operationalised by the Legal Services Authorities Act, 1987 through NALSA, state and district authorities, and trained para-legal volunteers.</t>
         </is>
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>AP's SSAAT recovered Rs. 400+ crore in misappropriated funds</t>
-        </is>
-      </c>
-      <c r="F43" s="9" t="inlineStr"/>
+          <t>A district legal services authority’s para-legal volunteers help MGNREGA workers file claims for unpaid wages and compensation for delayed payment.</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="n"/>
     </row>
     <row r="44" ht="45" customHeight="1">
       <c r="A44" s="2" t="n">
@@ -1765,27 +1741,27 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>PESA</t>
+          <t>Reservation Policy</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Rights-Based Legislation</t>
+          <t>Social Justice</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>Panchayats (Extension to Scheduled Areas) Act, 1996. Gram Sabha consent for land acquisition in Fifth Schedule areas.</t>
+          <t>Affirmative action under Articles 15(4), 16(4), and 243D for Scheduled Castes, Scheduled Tribes, Other Backward Classes, and women in education, public employment, and local bodies. Courts treat it as a facet of substantive equality, not an exception to it.</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>Gram Sabha power to approve/reject development projects in Scheduled Areas</t>
+          <t>Indra Sawhney (1992): 50% ceiling, creamy layer exclusion for OBCs</t>
         </is>
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>Fifth Schedule</t>
+          <t>Articles 15(4), 16(4)</t>
         </is>
       </c>
     </row>
@@ -1795,25 +1771,25 @@
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>BNS/BNSS/BSA</t>
+          <t>Creamy Layer</t>
         </is>
       </c>
       <c r="C45" s="8" t="inlineStr">
         <is>
-          <t>Criminal Justice</t>
+          <t>Social Justice</t>
         </is>
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>Bharatiya Nyaya Sanhita, Nagarik Suraksha Sanhita, Sakshya Adhiniyam (2023) replacing IPC, CrPC, Evidence Act. Effective July 2024.</t>
+          <t>Economic threshold above which OBC individuals excluded from reservation. Currently Rs. 8 lakh. Does not apply to SC/ST.</t>
         </is>
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>Community service as punishment, electronic evidence, zero FIR. Critics note many colonial provisions retained</t>
-        </is>
-      </c>
-      <c r="F45" s="9" t="inlineStr"/>
+          <t>Introduced in Indra Sawhney (1992) to ensure benefits reach most disadvantaged OBCs</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="n"/>
     </row>
     <row r="46" ht="45" customHeight="1">
       <c r="A46" s="2" t="n">
@@ -1821,27 +1797,27 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>Undertrial Crisis</t>
+          <t>EWS Reservation</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Criminal Justice</t>
+          <t>Social Justice</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>77% of 5+ lakh prisoners are undertrials. Many serve longer awaiting trial than maximum sentence for alleged offence.</t>
+          <t>10% for Economically Weaker Sections among unreserved categories. 103rd Amendment (2019). Upheld in Janhit Abhiyan (2022), 3:2.</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>Sec. 479 BNSS mandates release after half maximum sentence; implementation poor</t>
+          <t>First economic-only reservation in Indian constitutional history</t>
         </is>
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>Article 21, 22</t>
+          <t>Article 15(6), 16(6)</t>
         </is>
       </c>
     </row>
@@ -1851,29 +1827,25 @@
       </c>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>Custodial Violence</t>
+          <t>Sub-Classification of SCs</t>
         </is>
       </c>
       <c r="C47" s="8" t="inlineStr">
         <is>
-          <t>Criminal Justice</t>
+          <t>Social Justice</t>
         </is>
       </c>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>Torture or death in custody. D.K. Basu (1997) established mandatory guidelines: medical exam, inform family, arrest records.</t>
+          <t>States may create sub-categories within SCs for preferential treatment. Permitted in State of Punjab v. Davinder Singh (2024).</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>NHRC receives thousands of custodial death complaints annually. India has not ratified UNCAT</t>
-        </is>
-      </c>
-      <c r="F47" s="9" t="inlineStr">
-        <is>
-          <t>Article 21</t>
-        </is>
-      </c>
+          <t>Allows prioritizing Valmikis, Mazhabi Sikhs, Arunthathiyars within SC category</t>
+        </is>
+      </c>
+      <c r="F47" s="9" t="n"/>
     </row>
     <row r="48" ht="45" customHeight="1">
       <c r="A48" s="2" t="n">
@@ -1881,25 +1853,29 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>Police Reform</t>
+          <t>Political Reservation</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Criminal Justice</t>
+          <t>Social Justice</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>Prakash Singh v. UOI (2006): fixed DGP tenure, State Security Commissions, separation of investigation from law and order.</t>
+          <t>Reserved seats in Parliament and state legislatures for SC/ST proportional to population. Extended to 2030.</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>Most states only partially implemented; political control over transfers remains pervasive</t>
-        </is>
-      </c>
-      <c r="F48" s="5" t="inlineStr"/>
+          <t>Pande (2003, AER): increased targeted public goods spending in SC-reserved constituencies</t>
+        </is>
+      </c>
+      <c r="F48" s="5" t="inlineStr">
+        <is>
+          <t>Articles 330-333</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="45" customHeight="1">
       <c r="A49" s="6" t="n">
@@ -1907,29 +1883,25 @@
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>EIA Notification</t>
+          <t>RTI Act</t>
         </is>
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>Environmental Law</t>
+          <t>Rights-Based Legislation</t>
         </is>
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>Environmental Impact Assessment (2006) requires prior clearance for major projects through screening, scoping, public hearing, expert appraisal.</t>
+          <t>The law giving every citizen the right to information held by public authorities, with 30-day deadlines, penalties on erring officers, and Information Commissions in appeal. It grew out of the MKSS movement for wage records in rural Rajasthan.</t>
         </is>
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>Draft EIA 2020 proposed post-facto clearance; 2 million+ public comments opposing dilutions</t>
-        </is>
-      </c>
-      <c r="F49" s="9" t="inlineStr">
-        <is>
-          <t>EPA 1986</t>
-        </is>
-      </c>
+          <t>40-60 lakh applications annually. Peisakhin &amp; Pinto (2010): RTI reduced bureaucratic delays</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="n"/>
     </row>
     <row r="50" ht="45" customHeight="1">
       <c r="A50" s="2" t="n">
@@ -1937,27 +1909,27 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>NGT</t>
+          <t>MGNREGA</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>Environmental Law</t>
+          <t>Rights-Based Legislation</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>National Green Tribunal (2010). Specialized environmental court for civil cases on environmental protection and natural resources.</t>
+          <t>The Mahatma Gandhi National Rural Employment Guarantee Act, 2005 — a statutory guarantee of 100 days of wage work per rural household, on demand, with unemployment allowance if work is not provided. It is the paradigm of rights-based framing: a justiciable entitlement, not a scheme. The Act was repealed from 1 July 2026 and replaced by the Viksit Bharat G RAM G Act 2025, which raises the guarantee to 125 days.</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
         <is>
-          <t>Banned commercial activity near rivers, regulated eco-sensitive zones, imposed environmental compensation</t>
+          <t>Imbert &amp; Papp (2015, AER): raised private-sector wages by 4.7%. Muralidharan et al. (2016): biometrics reduced leakage 40%</t>
         </is>
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>NGT Act 2010</t>
+          <t>Article 41 (DPSP)</t>
         </is>
       </c>
     </row>
@@ -1967,29 +1939,25 @@
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>Polluter Pays Principle</t>
+          <t>Forest Rights Act</t>
         </is>
       </c>
       <c r="C51" s="8" t="inlineStr">
         <is>
-          <t>Environmental Law</t>
+          <t>Rights-Based Legislation</t>
         </is>
       </c>
       <c r="D51" s="9" t="inlineStr">
         <is>
-          <t>Cost of pollution borne by the entity causing it. Adopted in Vellore Citizens v. UOI (1996) alongside precautionary principle.</t>
+          <t>The law recognising individual and community rights of forest-dwelling Scheduled Tribes and other traditional forest dwellers over land and forest resources, with the Gram Sabha as the authority that initiates recognition. It reframes forest dwellers from encroachers to rights-holders.</t>
         </is>
       </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>Vellore tanneries ordered to pay compensation and remediation costs</t>
-        </is>
-      </c>
-      <c r="F51" s="9" t="inlineStr">
-        <is>
-          <t>Article 21</t>
-        </is>
-      </c>
+          <t>Section 4(5): Gram Sabha consent required before forest land diversion</t>
+        </is>
+      </c>
+      <c r="F51" s="9" t="n"/>
     </row>
     <row r="52" ht="45" customHeight="1">
       <c r="A52" s="2" t="n">
@@ -1997,27 +1965,27 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>Public Trust Doctrine</t>
+          <t>RTE Act</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Environmental Law</t>
+          <t>Rights-Based Legislation</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>State holds natural resources as trustee for the public. Adopted in M.C. Mehta v. Kamal Nath (1997).</t>
+          <t>The statute operationalising Article 21A: free and compulsory education for children aged 6-14, norms for schools, a 25% quota for disadvantaged children in private schools, and a ban on corporal punishment and board exams till elementary level.</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t>Prevented private encroachment on riverbed land; applied to village commons and water bodies</t>
+          <t>ASER 2023: near-universal enrollment but only 65% of Grade 5 children read Grade 2 text</t>
         </is>
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>Article 21</t>
+          <t>Article 21A</t>
         </is>
       </c>
     </row>
@@ -2027,27 +1995,27 @@
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>Absolute Liability</t>
+          <t>NFSA</t>
         </is>
       </c>
       <c r="C53" s="8" t="inlineStr">
         <is>
-          <t>Environmental Law</t>
+          <t>Rights-Based Legislation</t>
         </is>
       </c>
       <c r="D53" s="9" t="inlineStr">
         <is>
-          <t>Enterprises in inherently dangerous activities owe absolute duty of care. No defenses. M.C. Mehta v. UOI (1987, Oleum Gas Leak).</t>
+          <t>The law converting food programmes into legal entitlements: subsidised grain for two-thirds of the population, maternity benefits, and nutritional norms for ICDS and mid-day meals, with grievance redressal machinery.</t>
         </is>
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>Goes beyond British strict liability (Rylands v. Fletcher). Greater profit = greater compensation</t>
+          <t>Dreze &amp; Khera (2017): PDS reform improved delivery but created exclusion errors</t>
         </is>
       </c>
       <c r="F53" s="9" t="inlineStr">
         <is>
-          <t>Article 21</t>
+          <t>Article 47 (DPSP)</t>
         </is>
       </c>
     </row>
@@ -2057,29 +2025,25 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>Forest Conservation</t>
+          <t>Social Audit</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>Environmental Law</t>
+          <t>Rights-Based Legislation</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>FC Act (1980) requires central approval for forest land diversion. T.N. Godavarman (1996) expanded to all forests.</t>
+          <t>A statutory process of public verification of records and works by the community itself, mandated under Section 17 of MGNREGA and extended to other schemes; Meghalaya passed the first law making social audit compulsory across departments. It institutionalises the jan sunwai.</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t>CAMPA fund: Rs. 54,000+ crore accumulated, ~30% utilization. FC Amendment Act 2023 exempts certain categories</t>
-        </is>
-      </c>
-      <c r="F54" s="5" t="inlineStr">
-        <is>
-          <t>FCA 1980</t>
-        </is>
-      </c>
+          <t>AP's SSAAT recovered Rs. 400+ crore in misappropriated funds</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="n"/>
     </row>
     <row r="55" ht="45" customHeight="1">
       <c r="A55" s="6" t="n">
@@ -2087,27 +2051,27 @@
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>Precautionary Principle</t>
+          <t>PESA</t>
         </is>
       </c>
       <c r="C55" s="8" t="inlineStr">
         <is>
-          <t>Environmental Law</t>
+          <t>Rights-Based Legislation</t>
         </is>
       </c>
       <c r="D55" s="9" t="inlineStr">
         <is>
-          <t>Where serious environmental damage threatened, lack of scientific certainty does not justify postponing prevention. Vellore Citizens (1996).</t>
+          <t>The Panchayats (Extension to the Scheduled Areas) Act, extending panchayati raj to Fifth Schedule areas with special powers: Gram Sabha consultation on land acquisition, control over minor forest produce, minor minerals, and local plans. Its promise depends on state rules actually devolving these powers.</t>
         </is>
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>Burden of proof shifts to developer: proponent must prove safety, not opponents prove harm</t>
+          <t>Gram Sabha power to approve/reject development projects in Scheduled Areas</t>
         </is>
       </c>
       <c r="F55" s="9" t="inlineStr">
         <is>
-          <t>Article 21</t>
+          <t>Fifth Schedule</t>
         </is>
       </c>
     </row>
@@ -2117,29 +2081,25 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>Climate Litigation</t>
+          <t>LARR Act, 2013</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>Environmental Law</t>
+          <t>Rights-Based Legislation</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>Legal action invoking constitutional rights to address climate change. M.K. Ranjitsinh v. UOI (2024) recognized right under Arts. 14 &amp; 21.</t>
+          <t>The Right to Fair Compensation and Transparency in Land Acquisition, Rehabilitation and Resettlement Act, replacing the 1894 law: consent of 70-80% of affected families for PPP and private acquisitions, social impact assessment, and compensation up to four times market value in rural areas.</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t>Opens door to challenges against inadequate government action on emissions and climate adaptation</t>
-        </is>
-      </c>
-      <c r="F56" s="5" t="inlineStr">
-        <is>
-          <t>Articles 14, 21</t>
-        </is>
-      </c>
+          <t>A social impact assessment hearing under LARR gives displaced sharecroppers — not just titled owners — a documented claim to rehabilitation.</t>
+        </is>
+      </c>
+      <c r="F56" s="5" t="n"/>
     </row>
     <row r="57" ht="45" customHeight="1">
       <c r="A57" s="6" t="n">
@@ -2147,29 +2107,25 @@
       </c>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>Aadhaar</t>
+          <t>Street Vendors Act, 2014</t>
         </is>
       </c>
       <c r="C57" s="8" t="inlineStr">
         <is>
-          <t>Digital Rights</t>
+          <t>Rights-Based Legislation</t>
         </is>
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>12-digit biometric identity for 1.3+ billion residents. Puttaswamy (Aadhaar, 2018): upheld for subsidies, struck down Sec. 57 private use.</t>
+          <t>The law protecting urban vendors’ right to livelihood: surveys before eviction, vending certificates, Town Vending Committees with 40% vendor representation, and designated vending zones. It followed Supreme Court rulings recognising vending as a fundamental right under Article 19(1)(g).</t>
         </is>
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>Dreze &amp; Khera: authentication failures excluding elderly, manual laborers from PDS rations</t>
-        </is>
-      </c>
-      <c r="F57" s="9" t="inlineStr">
-        <is>
-          <t>Article 21</t>
-        </is>
-      </c>
+          <t>A vendors’ union uses the Act’s no-eviction-without-survey rule to stall a drive that would have confiscated carts before the town completed its vendor survey.</t>
+        </is>
+      </c>
+      <c r="F57" s="9" t="n"/>
     </row>
     <row r="58" ht="45" customHeight="1">
       <c r="A58" s="2" t="n">
@@ -2177,29 +2133,25 @@
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>DPDP Act</t>
+          <t>BNS/BNSS/BSA</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>Digital Rights</t>
+          <t>Criminal Justice</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>Digital Personal Data Protection Act (2023). Consent-based framework. Data Protection Board. Significant government exemptions.</t>
+          <t>Bharatiya Nyaya Sanhita, Nagarik Suraksha Sanhita, Sakshya Adhiniyam (2023) replacing IPC, CrPC, Evidence Act. Effective July 2024.</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t>Unlike GDPR: no data localization, no portability right. Government exemptions raise surveillance concerns</t>
-        </is>
-      </c>
-      <c r="F58" s="5" t="inlineStr">
-        <is>
-          <t>Article 21</t>
-        </is>
-      </c>
+          <t>Community service as punishment, electronic evidence, zero FIR. Critics note many colonial provisions retained</t>
+        </is>
+      </c>
+      <c r="F58" s="5" t="n"/>
     </row>
     <row r="59" ht="45" customHeight="1">
       <c r="A59" s="6" t="n">
@@ -2207,27 +2159,27 @@
       </c>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>Internet Shutdowns</t>
+          <t>Undertrial Crisis</t>
         </is>
       </c>
       <c r="C59" s="8" t="inlineStr">
         <is>
-          <t>Digital Rights</t>
+          <t>Criminal Justice</t>
         </is>
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>Government-ordered internet suspension. India leads globally (116 in 2022). Anuradha Bhasin (2020): must be proportionate, time-limited, published.</t>
+          <t>77% of 5+ lakh prisoners are undertrials. Many serve longer awaiting trial than maximum sentence for alleged offence.</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>Kashmir shutdown (Aug 2019-Mar 2020): longest in any democracy. Court held disproportionate</t>
+          <t>Sec. 479 BNSS mandates release after half maximum sentence; implementation poor</t>
         </is>
       </c>
       <c r="F59" s="9" t="inlineStr">
         <is>
-          <t>Article 19(1)(a), 21</t>
+          <t>Article 21, 22</t>
         </is>
       </c>
     </row>
@@ -2237,22 +2189,22 @@
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>Digital Public Infrastructure</t>
+          <t>Custodial Violence</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>Digital Rights</t>
+          <t>Criminal Justice</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>India Stack: Aadhaar (identity) + UPI (payments) + DigiLocker + Account Aggregator. G20-endorsed DPI model.</t>
+          <t>Torture or death in custody. D.K. Basu (1997) established mandatory guidelines: medical exam, inform family, arrest records.</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t>UPI: 13+ billion transactions/month. Constitutional questions about data governance without comprehensive privacy law</t>
+          <t>NHRC receives thousands of custodial death complaints annually. India has not ratified UNCAT</t>
         </is>
       </c>
       <c r="F60" s="5" t="inlineStr">
@@ -2267,29 +2219,25 @@
       </c>
       <c r="B61" s="7" t="inlineStr">
         <is>
-          <t>Right to Be Forgotten</t>
+          <t>Police Reform</t>
         </is>
       </c>
       <c r="C61" s="8" t="inlineStr">
         <is>
-          <t>Digital Rights</t>
+          <t>Criminal Justice</t>
         </is>
       </c>
       <c r="D61" s="9" t="inlineStr">
         <is>
-          <t>Right to have personal information removed from public access. Not explicit in DPDP Act but recognized by some High Courts.</t>
+          <t>Prakash Singh v. UOI (2006): fixed DGP tenure, State Security Commissions, separation of investigation from law and order.</t>
         </is>
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>Karnataka HC (2017): ordered name removal from criminal judgment after acquittal</t>
-        </is>
-      </c>
-      <c r="F61" s="9" t="inlineStr">
-        <is>
-          <t>Article 21</t>
-        </is>
-      </c>
+          <t>Most states only partially implemented; political control over transfers remains pervasive</t>
+        </is>
+      </c>
+      <c r="F61" s="9" t="n"/>
     </row>
     <row r="62" ht="45" customHeight="1">
       <c r="A62" s="2" t="n">
@@ -2297,25 +2245,29 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>Bangladesh Constitution</t>
+          <t>EIA Notification</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>Comparative South Asia</t>
+          <t>Environmental Law</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>1972 Constitution. Four pillars: nationalism, socialism, democracy, secularism. Basic structure doctrine: Anwar Hossain Chowdhury (1989).</t>
+          <t>Environmental Impact Assessment (2006) requires prior clearance for major projects through screening, scoping, public hearing, expert appraisal.</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t>2024 crisis: PM Hasina resigned, interim government under Yunus. Constitutional fragility when norms erode</t>
-        </is>
-      </c>
-      <c r="F62" s="5" t="inlineStr"/>
+          <t>Draft EIA 2020 proposed post-facto clearance; 2 million+ public comments opposing dilutions</t>
+        </is>
+      </c>
+      <c r="F62" s="5" t="inlineStr">
+        <is>
+          <t>EPA 1986</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="45" customHeight="1">
       <c r="A63" s="6" t="n">
@@ -2323,25 +2275,29 @@
       </c>
       <c r="B63" s="7" t="inlineStr">
         <is>
-          <t>Nepal Constitution</t>
+          <t>NGT</t>
         </is>
       </c>
       <c r="C63" s="8" t="inlineStr">
         <is>
-          <t>Comparative South Asia</t>
+          <t>Environmental Law</t>
         </is>
       </c>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>2015 Constitution: federal democratic republic, 31 fundamental rights, 7 provinces, proportional representation.</t>
+          <t>National Green Tribunal (2010). Specialized environmental court for civil cases on environmental protection and natural resources.</t>
         </is>
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>Includes justiciable socio-economic rights that India keeps as non-justiciable DPSPs</t>
-        </is>
-      </c>
-      <c r="F63" s="9" t="inlineStr"/>
+          <t>Banned commercial activity near rivers, regulated eco-sensitive zones, imposed environmental compensation</t>
+        </is>
+      </c>
+      <c r="F63" s="9" t="inlineStr">
+        <is>
+          <t>NGT Act 2010</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="45" customHeight="1">
       <c r="A64" s="2" t="n">
@@ -2349,25 +2305,29 @@
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>Sri Lanka Constitution</t>
+          <t>Polluter Pays Principle</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>Comparative South Asia</t>
+          <t>Environmental Law</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>1978 Constitution: executive presidential system. 21st Amendment (2022) restored parliamentary checks after Aragalaya crisis.</t>
+          <t>Cost of pollution borne by the entity causing it. Adopted in Vellore Citizens v. UOI (1996) alongside precautionary principle.</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t>2022 economic crisis showed how executive power concentration eliminated institutional checks</t>
-        </is>
-      </c>
-      <c r="F64" s="5" t="inlineStr"/>
+          <t>Vellore tanneries ordered to pay compensation and remediation costs</t>
+        </is>
+      </c>
+      <c r="F64" s="5" t="inlineStr">
+        <is>
+          <t>Article 21</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="45" customHeight="1">
       <c r="A65" s="6" t="n">
@@ -2375,25 +2335,29 @@
       </c>
       <c r="B65" s="7" t="inlineStr">
         <is>
-          <t>Pakistan Constitution</t>
+          <t>Public Trust Doctrine</t>
         </is>
       </c>
       <c r="C65" s="8" t="inlineStr">
         <is>
-          <t>Comparative South Asia</t>
+          <t>Environmental Law</t>
         </is>
       </c>
       <c r="D65" s="9" t="inlineStr">
         <is>
-          <t>1973 Constitution: federal parliamentary democracy with Islamic provisions. 18th Amendment (2010) decentralized 47 subjects to provinces.</t>
+          <t>The doctrine that the state holds natural resources — rivers, lakes, forests, air — in trust for the public and cannot alienate them for private gain in breach of that trust. Indian courts imported it into environmental jurisprudence under Article 21.</t>
         </is>
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>18th Amendment abolished Concurrent List entirely, most significant devolution in Pakistan's history</t>
-        </is>
-      </c>
-      <c r="F65" s="9" t="inlineStr"/>
+          <t>Prevented private encroachment on riverbed land; applied to village commons and water bodies</t>
+        </is>
+      </c>
+      <c r="F65" s="9" t="inlineStr">
+        <is>
+          <t>Article 21</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="45" customHeight="1">
       <c r="A66" s="2" t="n">
@@ -2401,32 +2365,848 @@
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
+          <t>Absolute Liability</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>Environmental Law</t>
+        </is>
+      </c>
+      <c r="D66" s="5" t="inlineStr">
+        <is>
+          <t>Enterprises in inherently dangerous activities owe absolute duty of care. No defenses. M.C. Mehta v. UOI (1987, Oleum Gas Leak).</t>
+        </is>
+      </c>
+      <c r="E66" s="5" t="inlineStr">
+        <is>
+          <t>Goes beyond British strict liability (Rylands v. Fletcher). Greater profit = greater compensation</t>
+        </is>
+      </c>
+      <c r="F66" s="5" t="inlineStr">
+        <is>
+          <t>Article 21</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="45" customHeight="1">
+      <c r="A67" s="6" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" s="7" t="inlineStr">
+        <is>
+          <t>Forest Conservation</t>
+        </is>
+      </c>
+      <c r="C67" s="8" t="inlineStr">
+        <is>
+          <t>Environmental Law</t>
+        </is>
+      </c>
+      <c r="D67" s="9" t="inlineStr">
+        <is>
+          <t>FC Act (1980) requires central approval for forest land diversion. T.N. Godavarman (1996) expanded to all forests.</t>
+        </is>
+      </c>
+      <c r="E67" s="9" t="inlineStr">
+        <is>
+          <t>CAMPA fund: Rs. 54,000+ crore accumulated, ~30% utilization. FC Amendment Act 2023 exempts certain categories</t>
+        </is>
+      </c>
+      <c r="F67" s="9" t="inlineStr">
+        <is>
+          <t>FCA 1980</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="45" customHeight="1">
+      <c r="A68" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>Precautionary Principle</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>Environmental Law</t>
+        </is>
+      </c>
+      <c r="D68" s="5" t="inlineStr">
+        <is>
+          <t>Where serious environmental damage threatened, lack of scientific certainty does not justify postponing prevention. Vellore Citizens (1996).</t>
+        </is>
+      </c>
+      <c r="E68" s="5" t="inlineStr">
+        <is>
+          <t>Burden of proof shifts to developer: proponent must prove safety, not opponents prove harm</t>
+        </is>
+      </c>
+      <c r="F68" s="5" t="inlineStr">
+        <is>
+          <t>Article 21</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="45" customHeight="1">
+      <c r="A69" s="6" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" s="7" t="inlineStr">
+        <is>
+          <t>Climate Litigation</t>
+        </is>
+      </c>
+      <c r="C69" s="8" t="inlineStr">
+        <is>
+          <t>Environmental Law</t>
+        </is>
+      </c>
+      <c r="D69" s="9" t="inlineStr">
+        <is>
+          <t>Legal action invoking constitutional rights to address climate change. M.K. Ranjitsinh v. UOI (2024) recognized right under Arts. 14 &amp; 21.</t>
+        </is>
+      </c>
+      <c r="E69" s="9" t="inlineStr">
+        <is>
+          <t>Opens door to challenges against inadequate government action on emissions and climate adaptation</t>
+        </is>
+      </c>
+      <c r="F69" s="9" t="inlineStr">
+        <is>
+          <t>Articles 14, 21</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="45" customHeight="1">
+      <c r="A70" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>Aadhaar</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>Digital Rights</t>
+        </is>
+      </c>
+      <c r="D70" s="5" t="inlineStr">
+        <is>
+          <t>12-digit biometric identity for 1.3+ billion residents. Puttaswamy (Aadhaar, 2018): upheld for subsidies, struck down Sec. 57 private use.</t>
+        </is>
+      </c>
+      <c r="E70" s="5" t="inlineStr">
+        <is>
+          <t>Dreze &amp; Khera: authentication failures excluding elderly, manual laborers from PDS rations</t>
+        </is>
+      </c>
+      <c r="F70" s="5" t="inlineStr">
+        <is>
+          <t>Article 21</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="45" customHeight="1">
+      <c r="A71" s="6" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" s="7" t="inlineStr">
+        <is>
+          <t>DPDP Act</t>
+        </is>
+      </c>
+      <c r="C71" s="8" t="inlineStr">
+        <is>
+          <t>Digital Rights</t>
+        </is>
+      </c>
+      <c r="D71" s="9" t="inlineStr">
+        <is>
+          <t>The Digital Personal Data Protection Act, India’s first comprehensive data protection law: consent-based processing, obligations on data fiduciaries, special protections for children’s data, and penalties running to hundreds of crores. NGOs holding beneficiary databases are covered.</t>
+        </is>
+      </c>
+      <c r="E71" s="9" t="inlineStr">
+        <is>
+          <t>Unlike GDPR: no data localization, no portability right. Government exemptions raise surveillance concerns</t>
+        </is>
+      </c>
+      <c r="F71" s="9" t="inlineStr">
+        <is>
+          <t>Article 21</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="45" customHeight="1">
+      <c r="A72" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>Internet Shutdowns</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t>Digital Rights</t>
+        </is>
+      </c>
+      <c r="D72" s="5" t="inlineStr">
+        <is>
+          <t>Government-ordered internet suspension. India leads globally (116 in 2022). Anuradha Bhasin (2020): must be proportionate, time-limited, published.</t>
+        </is>
+      </c>
+      <c r="E72" s="5" t="inlineStr">
+        <is>
+          <t>Kashmir shutdown (Aug 2019-Mar 2020): longest in any democracy. Court held disproportionate</t>
+        </is>
+      </c>
+      <c r="F72" s="5" t="inlineStr">
+        <is>
+          <t>Article 19(1)(a), 21</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="45" customHeight="1">
+      <c r="A73" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" s="7" t="inlineStr">
+        <is>
+          <t>Digital Public Infrastructure</t>
+        </is>
+      </c>
+      <c r="C73" s="8" t="inlineStr">
+        <is>
+          <t>Digital Rights</t>
+        </is>
+      </c>
+      <c r="D73" s="9" t="inlineStr">
+        <is>
+          <t>India Stack: Aadhaar (identity) + UPI (payments) + DigiLocker + Account Aggregator. G20-endorsed DPI model.</t>
+        </is>
+      </c>
+      <c r="E73" s="9" t="inlineStr">
+        <is>
+          <t>UPI: 13+ billion transactions/month. Constitutional questions about data governance without comprehensive privacy law</t>
+        </is>
+      </c>
+      <c r="F73" s="9" t="inlineStr">
+        <is>
+          <t>Article 21</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="45" customHeight="1">
+      <c r="A74" s="2" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>Right to Be Forgotten</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t>Digital Rights</t>
+        </is>
+      </c>
+      <c r="D74" s="5" t="inlineStr">
+        <is>
+          <t>Right to have personal information removed from public access. Not explicit in DPDP Act but recognized by some High Courts.</t>
+        </is>
+      </c>
+      <c r="E74" s="5" t="inlineStr">
+        <is>
+          <t>Karnataka HC (2017): ordered name removal from criminal judgment after acquittal</t>
+        </is>
+      </c>
+      <c r="F74" s="5" t="inlineStr">
+        <is>
+          <t>Article 21</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="45" customHeight="1">
+      <c r="A75" s="6" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" s="7" t="inlineStr">
+        <is>
+          <t>Bangladesh Constitution</t>
+        </is>
+      </c>
+      <c r="C75" s="8" t="inlineStr">
+        <is>
+          <t>Comparative South Asia</t>
+        </is>
+      </c>
+      <c r="D75" s="9" t="inlineStr">
+        <is>
+          <t>1972 Constitution. Four pillars: nationalism, socialism, democracy, secularism. Basic structure doctrine: Anwar Hossain Chowdhury (1989).</t>
+        </is>
+      </c>
+      <c r="E75" s="9" t="inlineStr">
+        <is>
+          <t>2024 crisis: PM Hasina resigned, interim government under Yunus. Constitutional fragility when norms erode</t>
+        </is>
+      </c>
+      <c r="F75" s="9" t="n"/>
+    </row>
+    <row r="76" ht="45" customHeight="1">
+      <c r="A76" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>Nepal Constitution</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>Comparative South Asia</t>
+        </is>
+      </c>
+      <c r="D76" s="5" t="inlineStr">
+        <is>
+          <t>2015 Constitution: federal democratic republic, 31 fundamental rights, 7 provinces, proportional representation.</t>
+        </is>
+      </c>
+      <c r="E76" s="5" t="inlineStr">
+        <is>
+          <t>Includes justiciable socio-economic rights that India keeps as non-justiciable DPSPs</t>
+        </is>
+      </c>
+      <c r="F76" s="5" t="n"/>
+    </row>
+    <row r="77" ht="45" customHeight="1">
+      <c r="A77" s="6" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" s="7" t="inlineStr">
+        <is>
+          <t>Sri Lanka Constitution</t>
+        </is>
+      </c>
+      <c r="C77" s="8" t="inlineStr">
+        <is>
+          <t>Comparative South Asia</t>
+        </is>
+      </c>
+      <c r="D77" s="9" t="inlineStr">
+        <is>
+          <t>1978 Constitution: executive presidential system. 21st Amendment (2022) restored parliamentary checks after Aragalaya crisis.</t>
+        </is>
+      </c>
+      <c r="E77" s="9" t="inlineStr">
+        <is>
+          <t>2022 economic crisis showed how executive power concentration eliminated institutional checks</t>
+        </is>
+      </c>
+      <c r="F77" s="9" t="n"/>
+    </row>
+    <row r="78" ht="45" customHeight="1">
+      <c r="A78" s="2" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>Pakistan Constitution</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t>Comparative South Asia</t>
+        </is>
+      </c>
+      <c r="D78" s="5" t="inlineStr">
+        <is>
+          <t>1973 Constitution: federal parliamentary democracy with Islamic provisions. 18th Amendment (2010) decentralized 47 subjects to provinces.</t>
+        </is>
+      </c>
+      <c r="E78" s="5" t="inlineStr">
+        <is>
+          <t>18th Amendment abolished Concurrent List entirely, most significant devolution in Pakistan's history</t>
+        </is>
+      </c>
+      <c r="F78" s="5" t="n"/>
+    </row>
+    <row r="79" ht="45" customHeight="1">
+      <c r="A79" s="6" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" s="7" t="inlineStr">
+        <is>
           <t>Asymmetric Federalism</t>
         </is>
       </c>
-      <c r="C66" s="4" t="inlineStr">
+      <c r="C79" s="8" t="inlineStr">
         <is>
           <t>Comparative South Asia</t>
         </is>
       </c>
-      <c r="D66" s="5" t="inlineStr">
+      <c r="D79" s="9" t="inlineStr">
         <is>
           <t>Different constituent units have different autonomy levels. India: Arts. 370 (abrogated), 371A-J, Fifth and Sixth Schedules.</t>
         </is>
       </c>
-      <c r="E66" s="5" t="inlineStr">
+      <c r="E79" s="9" t="inlineStr">
         <is>
           <t>Nagaland Art. 371A: national legislation may not apply without state legislature consent on customary law</t>
         </is>
       </c>
-      <c r="F66" s="5" t="inlineStr">
+      <c r="F79" s="9" t="inlineStr">
         <is>
           <t>Articles 370, 371A-J</t>
         </is>
       </c>
     </row>
+    <row r="80" ht="45" customHeight="1">
+      <c r="A80" s="2" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>POSH Act, 2013</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>Protection &amp; Welfare Laws</t>
+        </is>
+      </c>
+      <c r="D80" s="5" t="inlineStr">
+        <is>
+          <t>The Sexual Harassment of Women at Workplace (Prevention, Prohibition and Redressal) Act, codifying the Vishaka guidelines: Internal Committees in workplaces with 10 or more employees, Local Committees for smaller and informal workplaces, and time-bound inquiries.</t>
+        </is>
+      </c>
+      <c r="E80" s="5" t="inlineStr">
+        <is>
+          <t>The Act exists because Vishaka v State of Rajasthan (1997) — filed after the gang rape of saathin Bhanwari Devi — made the Supreme Court legislate interim guidelines; every NGO with ten staff must now have an Internal Committee.</t>
+        </is>
+      </c>
+      <c r="F80" s="5" t="n"/>
+    </row>
+    <row r="81" ht="45" customHeight="1">
+      <c r="A81" s="6" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" s="7" t="inlineStr">
+        <is>
+          <t>Juvenile Justice Act, 2015</t>
+        </is>
+      </c>
+      <c r="C81" s="8" t="inlineStr">
+        <is>
+          <t>Protection &amp; Welfare Laws</t>
+        </is>
+      </c>
+      <c r="D81" s="9" t="inlineStr">
+        <is>
+          <t>The framework for children in conflict with the law and children in need of care and protection: Juvenile Justice Boards, Child Welfare Committees, registered child-care institutions, and adoption through CARA. It prioritises rehabilitation over punishment.</t>
+        </is>
+      </c>
+      <c r="E81" s="9" t="inlineStr">
+        <is>
+          <t>A child rescued from a bangle workshop is produced before the Child Welfare Committee, which orders shelter, schooling, and repatriation — the statutory pipeline child-rights NGOs work within.</t>
+        </is>
+      </c>
+      <c r="F81" s="9" t="n"/>
+    </row>
+    <row r="82" ht="45" customHeight="1">
+      <c r="A82" s="2" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>POCSO Act, 2012</t>
+        </is>
+      </c>
+      <c r="C82" s="4" t="inlineStr">
+        <is>
+          <t>Protection &amp; Welfare Laws</t>
+        </is>
+      </c>
+      <c r="D82" s="5" t="inlineStr">
+        <is>
+          <t>The Protection of Children from Sexual Offences Act: gender-neutral offences, child-friendly recording of evidence, special courts, and mandatory reporting of suspected abuse by any person, including NGO staff and teachers.</t>
+        </is>
+      </c>
+      <c r="E82" s="5" t="inlineStr">
+        <is>
+          <t>A school counsellor who learns of abuse is legally bound to report it to police or the CWC — failure to report is itself an offence, a duty frontline training must cover.</t>
+        </is>
+      </c>
+      <c r="F82" s="5" t="n"/>
+    </row>
+    <row r="83" ht="45" customHeight="1">
+      <c r="A83" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" s="7" t="inlineStr">
+        <is>
+          <t>Domestic Violence Act, 2005</t>
+        </is>
+      </c>
+      <c r="C83" s="8" t="inlineStr">
+        <is>
+          <t>Protection &amp; Welfare Laws</t>
+        </is>
+      </c>
+      <c r="D83" s="9" t="inlineStr">
+        <is>
+          <t>The Protection of Women from Domestic Violence Act — a civil law giving women protection orders, residence orders, monetary relief, and custody orders, enforced through Protection Officers, without requiring a criminal prosecution. It covers all women in a shared household, including mothers and sisters.</t>
+        </is>
+      </c>
+      <c r="E83" s="9" t="inlineStr">
+        <is>
+          <t>A counselling centre helps a woman obtain a residence order so she cannot be thrown out of her marital home while maintenance proceedings continue.</t>
+        </is>
+      </c>
+      <c r="F83" s="9" t="n"/>
+    </row>
+    <row r="84" ht="45" customHeight="1">
+      <c r="A84" s="2" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>SC/ST (Prevention of Atrocities) Act, 1989</t>
+        </is>
+      </c>
+      <c r="C84" s="4" t="inlineStr">
+        <is>
+          <t>Protection &amp; Welfare Laws</t>
+        </is>
+      </c>
+      <c r="D84" s="5" t="inlineStr">
+        <is>
+          <t>The law criminalising caste-based atrocities with special courts, mandatory relief and rehabilitation for victims, and duties on officials — dereliction by public servants is itself punishable. Amendments in 2015 broadened offences to include social and economic boycotts.</t>
+        </is>
+      </c>
+      <c r="E84" s="5" t="inlineStr">
+        <is>
+          <t>After a Dalit groom is attacked for riding a horse, a legal-aid group ensures the FIR invokes the Atrocities Act so the family receives statutory relief and the case goes to a special court.</t>
+        </is>
+      </c>
+      <c r="F84" s="5" t="n"/>
+    </row>
+    <row r="85" ht="45" customHeight="1">
+      <c r="A85" s="6" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" s="7" t="inlineStr">
+        <is>
+          <t>Rights of Persons with Disabilities Act, 2016</t>
+        </is>
+      </c>
+      <c r="C85" s="8" t="inlineStr">
+        <is>
+          <t>Protection &amp; Welfare Laws</t>
+        </is>
+      </c>
+      <c r="D85" s="9" t="inlineStr">
+        <is>
+          <t>The law implementing the UN CRPD: 21 recognised disabilities, reasonable accommodation as a legal right, 4% reservation in government jobs, 5% in higher education, and accessibility obligations for public buildings and services.</t>
+        </is>
+      </c>
+      <c r="E85" s="9" t="inlineStr">
+        <is>
+          <t>A disability rights group uses the Act’s accessibility mandate to get ramps and accessible toilets included in a district’s school infrastructure plan rather than treated as optional add-ons.</t>
+        </is>
+      </c>
+      <c r="F85" s="9" t="n"/>
+    </row>
+    <row r="86" ht="45" customHeight="1">
+      <c r="A86" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>Bonded Labour System (Abolition) Act, 1976</t>
+        </is>
+      </c>
+      <c r="C86" s="4" t="inlineStr">
+        <is>
+          <t>Protection &amp; Welfare Laws</t>
+        </is>
+      </c>
+      <c r="D86" s="5" t="inlineStr">
+        <is>
+          <t>The law abolishing bonded labour and extinguishing all bonded debts, with District Magistrates responsible for identification, release, and rehabilitation. Release certificates trigger cash and non-cash rehabilitation entitlements.</t>
+        </is>
+      </c>
+      <c r="E86" s="5" t="inlineStr">
+        <is>
+          <t>Bandhua Mukti Morcha v Union of India (1984) — a letter treated as a PIL — forced the identification and release of bonded workers in Faridabad stone quarries and remains the template for release operations.</t>
+        </is>
+      </c>
+      <c r="F86" s="5" t="n"/>
+    </row>
+    <row r="87" ht="45" customHeight="1">
+      <c r="A87" s="6" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" s="7" t="inlineStr">
+        <is>
+          <t>Child Labour Act, 1986</t>
+        </is>
+      </c>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>Protection &amp; Welfare Laws</t>
+        </is>
+      </c>
+      <c r="D87" s="9" t="inlineStr">
+        <is>
+          <t>The Child and Adolescent Labour (Prohibition and Regulation) Act, which after the 2016 amendment bans all work by children under 14 (with a contested family-enterprise exception) and hazardous work for adolescents under 18. It links rescued children to rehabilitation funds and education.</t>
+        </is>
+      </c>
+      <c r="E87" s="9" t="inlineStr">
+        <is>
+          <t>A raid on a zari workshop invokes the Act alongside the JJ Act, and back wages plus fines feed the district child labour rehabilitation fund for the rescued children.</t>
+        </is>
+      </c>
+      <c r="F87" s="9" t="n"/>
+    </row>
+    <row r="88" ht="45" customHeight="1">
+      <c r="A88" s="2" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>FCRA, 2010</t>
+        </is>
+      </c>
+      <c r="C88" s="4" t="inlineStr">
+        <is>
+          <t>NGO Compliance &amp; Regulation</t>
+        </is>
+      </c>
+      <c r="D88" s="5" t="inlineStr">
+        <is>
+          <t>The Foreign Contribution (Regulation) Act, governing receipt of foreign funds by NGOs: registration or prior permission, a designated SBI New Delhi account, and, after the 2020 amendments, a ban on sub-granting to other organisations and a 20% cap on administrative expenses.</t>
+        </is>
+      </c>
+      <c r="E88" s="5" t="inlineStr">
+        <is>
+          <t>A grassroots organisation without FCRA registration cannot legally receive a foreign foundation’s grant even through an FCRA-registered intermediary — the 2020 sub-granting ban closed that route.</t>
+        </is>
+      </c>
+      <c r="F88" s="5" t="n"/>
+    </row>
+    <row r="89" ht="45" customHeight="1">
+      <c r="A89" s="6" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" s="7" t="inlineStr">
+        <is>
+          <t>Trust, Society, Section 8 Company</t>
+        </is>
+      </c>
+      <c r="C89" s="8" t="inlineStr">
+        <is>
+          <t>NGO Compliance &amp; Regulation</t>
+        </is>
+      </c>
+      <c r="D89" s="9" t="inlineStr">
+        <is>
+          <t>The three legal forms Indian nonprofits take: public charitable trusts (state trust laws), societies (Societies Registration Act, 1860), and Section 8 companies (Companies Act, 2013). They differ in governance rigour, compliance burden, and credibility with institutional funders.</t>
+        </is>
+      </c>
+      <c r="E89" s="9" t="inlineStr">
+        <is>
+          <t>A collective formalising for CSR funding often chooses a Section 8 company because corporate donors trust its audited, board-governed structure over an informal society.</t>
+        </is>
+      </c>
+      <c r="F89" s="9" t="n"/>
+    </row>
+    <row r="90" ht="45" customHeight="1">
+      <c r="A90" s="2" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>12A and 80G Registration</t>
+        </is>
+      </c>
+      <c r="C90" s="4" t="inlineStr">
+        <is>
+          <t>NGO Compliance &amp; Regulation</t>
+        </is>
+      </c>
+      <c r="D90" s="5" t="inlineStr">
+        <is>
+          <t>Income-tax registrations without which nonprofit status means little: 12A (now 12AB) exempts the organisation’s income from tax, and 80G lets donors claim deductions. Both now require periodic renewal and are linked to filing discipline.</t>
+        </is>
+      </c>
+      <c r="E90" s="5" t="inlineStr">
+        <is>
+          <t>A small NGO that missed its 12AB renewal window found its grant income treated as taxable — a compliance lapse that consumed a year of fundraising.</t>
+        </is>
+      </c>
+      <c r="F90" s="5" t="n"/>
+    </row>
+    <row r="91" ht="45" customHeight="1">
+      <c r="A91" s="6" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" s="7" t="inlineStr">
+        <is>
+          <t>CSR Mandate</t>
+        </is>
+      </c>
+      <c r="C91" s="8" t="inlineStr">
+        <is>
+          <t>NGO Compliance &amp; Regulation</t>
+        </is>
+      </c>
+      <c r="D91" s="9" t="inlineStr">
+        <is>
+          <t>Section 135 of the Companies Act, 2013, requiring qualifying companies to spend 2% of average net profits on activities listed in Schedule VII, with unspent amounts transferred to designated funds. Implementing NGOs must register with the MCA (Form CSR-1).</t>
+        </is>
+      </c>
+      <c r="E91" s="9" t="inlineStr">
+        <is>
+          <t>An education nonprofit registers on the CSR portal and aligns its proposal language to Schedule VII heads so a manufacturer’s CSR committee can legally fund its learning centres.</t>
+        </is>
+      </c>
+      <c r="F91" s="9" t="n"/>
+    </row>
+    <row r="92" ht="45" customHeight="1">
+      <c r="A92" s="2" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>Delegated Legislation</t>
+        </is>
+      </c>
+      <c r="C92" s="4" t="inlineStr">
+        <is>
+          <t>Legal Concepts &amp; Doctrine</t>
+        </is>
+      </c>
+      <c r="D92" s="5" t="inlineStr">
+        <is>
+          <t>Rules, notifications, schemes, and circulars made by the executive under powers delegated by a parent Act. Most of what practitioners experience as ‘the law’ — wage rates, eligibility criteria, forms — lives here, and it changes without Parliament.</t>
+        </is>
+      </c>
+      <c r="E92" s="5" t="inlineStr">
+        <is>
+          <t>MGNREGA wage rates are set by executive notification under Section 6, which is why wage campaigns target the rural development ministry’s notifications, not an amendment to the Act.</t>
+        </is>
+      </c>
+      <c r="F92" s="5" t="n"/>
+    </row>
+    <row r="93" ht="45" customHeight="1">
+      <c r="A93" s="6" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" s="7" t="inlineStr">
+        <is>
+          <t>Precedent</t>
+        </is>
+      </c>
+      <c r="C93" s="8" t="inlineStr">
+        <is>
+          <t>Legal Concepts &amp; Doctrine</t>
+        </is>
+      </c>
+      <c r="D93" s="9" t="inlineStr">
+        <is>
+          <t>The doctrine of stare decisis: courts follow earlier decisions on the same legal question, and under Article 141 the law declared by the Supreme Court binds all courts in India. High Court rulings bind within their state, which is why the same scheme can be run differently across states.</t>
+        </is>
+      </c>
+      <c r="E93" s="9" t="inlineStr">
+        <is>
+          <t>Once the Supreme Court held in PUCL that mid-day meals must be cooked, every state government was bound — one judgment changed school kitchens nationwide.</t>
+        </is>
+      </c>
+      <c r="F93" s="9" t="n"/>
+    </row>
+    <row r="94" ht="45" customHeight="1">
+      <c r="A94" s="2" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>Ultra Vires</t>
+        </is>
+      </c>
+      <c r="C94" s="4" t="inlineStr">
+        <is>
+          <t>Legal Concepts &amp; Doctrine</t>
+        </is>
+      </c>
+      <c r="D94" s="5" t="inlineStr">
+        <is>
+          <t>Literally ‘beyond powers’: an act of an authority or a piece of delegated legislation is void if it exceeds the powers conferred by the parent statute or the Constitution. It is the standard ground for challenging restrictive rules and circulars.</t>
+        </is>
+      </c>
+      <c r="E94" s="5" t="inlineStr">
+        <is>
+          <t>Activists challenge a state circular imposing conditions on ration eligibility that the NFSA nowhere authorises, arguing the circular is ultra vires the parent Act.</t>
+        </is>
+      </c>
+      <c r="F94" s="5" t="n"/>
+    </row>
+    <row r="95" ht="45" customHeight="1">
+      <c r="A95" s="6" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" s="7" t="inlineStr">
+        <is>
+          <t>Quasi-Judicial Bodies</t>
+        </is>
+      </c>
+      <c r="C95" s="8" t="inlineStr">
+        <is>
+          <t>Legal Concepts &amp; Doctrine</t>
+        </is>
+      </c>
+      <c r="D95" s="9" t="inlineStr">
+        <is>
+          <t>Authorities outside regular courts that decide rights after hearing parties — Information Commissions, the National Green Tribunal, consumer commissions, welfare boards. They are faster and cheaper than courts but their orders still bind and are appealable.</t>
+        </is>
+      </c>
+      <c r="E95" s="9" t="inlineStr">
+        <is>
+          <t>The National Green Tribunal ordered a halt to illegal sand mining on a riverbed within months — relief that would have taken years in a civil court.</t>
+        </is>
+      </c>
+      <c r="F95" s="9" t="n"/>
+    </row>
+    <row r="96" ht="45" customHeight="1">
+      <c r="A96" s="2" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>Statutory Commissions</t>
+        </is>
+      </c>
+      <c r="C96" s="4" t="inlineStr">
+        <is>
+          <t>Legal Concepts &amp; Doctrine</t>
+        </is>
+      </c>
+      <c r="D96" s="5" t="inlineStr">
+        <is>
+          <t>Bodies like the NHRC, State Human Rights Commissions, NCPCR, NCW, and the SC/ST Commissions, created by statute or the Constitution to inquire into violations, summon officials, and recommend action. Their powers are largely recommendatory, so their value depends on public pressure around their findings.</t>
+        </is>
+      </c>
+      <c r="E96" s="5" t="inlineStr">
+        <is>
+          <t>A child-rights group files a complaint before the NCPCR about children working in mica mines, using the Commission’s inquiry report to push the district administration into rescue and enrolment drives.</t>
+        </is>
+      </c>
+      <c r="F96" s="5" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F66"/>
+  <autoFilter ref="A1:F96"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2437,7 +3217,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2484,7 +3264,7 @@
         </is>
       </c>
       <c r="B3" s="12" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C3" s="13" t="inlineStr">
         <is>
@@ -2544,7 +3324,7 @@
         </is>
       </c>
       <c r="B7" s="12" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C7" s="13" t="inlineStr">
         <is>
@@ -2559,7 +3339,7 @@
         </is>
       </c>
       <c r="B8" s="12" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="C8" s="13" t="inlineStr">
         <is>
@@ -2570,43 +3350,88 @@
     <row r="9">
       <c r="A9" s="11" t="inlineStr">
         <is>
-          <t>Rights-Based Legislation</t>
+          <t>Legal Concepts &amp; Doctrine</t>
         </is>
       </c>
       <c r="B9" s="12" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C9" s="13" t="inlineStr">
         <is>
-          <t>RTI, MGNREGA, FRA, RTE, NFSA, PESA, social audits with implementation data and academic research</t>
+          <t>Delegated legislation, precedent, ultra vires, quasi-judicial bodies, statutory commissions</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>Social Justice</t>
+          <t>NGO Compliance &amp; Regulation</t>
         </is>
       </c>
       <c r="B10" s="12" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C10" s="13" t="inlineStr">
         <is>
-          <t>Reservation policy, creamy layer, EWS, sub-classification, political reservation with empirical evidence (Pande, Chattopadhyay &amp; Duflo)</t>
+          <t>FCRA, nonprofit legal forms (trust, society, Section 8 company), 12A and 80G registration, CSR mandate</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
         <is>
-          <t>State Policy &amp; Governance</t>
+          <t>Protection &amp; Welfare Laws</t>
         </is>
       </c>
       <c r="B11" s="12" t="n">
         <v>8</v>
       </c>
       <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>POSH, Juvenile Justice, POCSO, Domestic Violence, SC/ST (Prevention of Atrocities), Rights of Persons with Disabilities, Bonded Labour and Child Labour Acts</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>Rights-Based Legislation</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>RTI, MGNREGA, FRA, RTE, NFSA, PESA, social audits with implementation data and academic research</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>Social Justice</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>Reservation policy, creamy layer, EWS, sub-classification, political reservation with empirical evidence (Pande, Chattopadhyay &amp; Duflo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>State Policy &amp; Governance</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
         <is>
           <t>DPSPs, governance frameworks: panchayati raj, fiscal federalism, Finance Commission, President's Rule, anti-defection, fundamental duties</t>
         </is>

</xml_diff>